<commit_message>
UPDATE: company data infomrmation - added new company
</commit_message>
<xml_diff>
--- a/data/eko_transaction.xlsx
+++ b/data/eko_transaction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3ACBADD-125D-4407-BAC4-717EB3611514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C839D2C-FAAD-4B79-924C-DBE26A321516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED1E34D5-CC3F-4E59-90C6-24BBB446287E}"/>
   </bookViews>
@@ -6011,7 +6011,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6030,6 +6030,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -6043,7 +6049,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -6052,6 +6058,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6401,7 +6408,7 @@
     <col min="16" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="32" customWidth="1"/>
     <col min="22" max="22" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="8.42578125" bestFit="1" customWidth="1"/>
@@ -58136,10 +58143,10 @@
       <c r="T672" s="1" t="s">
         <v>1160</v>
       </c>
-      <c r="U672" s="1" t="s">
+      <c r="U672" s="6" t="s">
         <v>1161</v>
       </c>
-      <c r="V672" s="1" t="s">
+      <c r="V672" s="6" t="s">
         <v>1162</v>
       </c>
       <c r="W672" s="1" t="s">
@@ -58290,10 +58297,10 @@
       <c r="T674" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="U674" s="1" t="s">
+      <c r="U674" s="6" t="s">
         <v>1167</v>
       </c>
-      <c r="V674" s="1" t="s">
+      <c r="V674" s="6" t="s">
         <v>1168</v>
       </c>
       <c r="W674" s="1" t="s">
@@ -58367,10 +58374,10 @@
       <c r="T675" s="1" t="s">
         <v>1171</v>
       </c>
-      <c r="U675" s="1" t="s">
+      <c r="U675" s="6" t="s">
         <v>1172</v>
       </c>
-      <c r="V675" s="1" t="s">
+      <c r="V675" s="6" t="s">
         <v>1173</v>
       </c>
       <c r="W675" s="1" t="s">
@@ -58444,10 +58451,10 @@
       <c r="T676" s="1" t="s">
         <v>1176</v>
       </c>
-      <c r="U676" s="1" t="s">
+      <c r="U676" s="6" t="s">
         <v>1177</v>
       </c>
-      <c r="V676" s="1" t="s">
+      <c r="V676" s="6" t="s">
         <v>1178</v>
       </c>
       <c r="W676" s="1" t="s">
@@ -58521,10 +58528,10 @@
       <c r="T677" s="1" t="s">
         <v>1181</v>
       </c>
-      <c r="U677" s="1" t="s">
+      <c r="U677" s="6" t="s">
         <v>1182</v>
       </c>
-      <c r="V677" s="1" t="s">
+      <c r="V677" s="6" t="s">
         <v>1183</v>
       </c>
       <c r="W677" s="1" t="s">
@@ -58598,10 +58605,10 @@
       <c r="T678" s="1" t="s">
         <v>644</v>
       </c>
-      <c r="U678" s="1" t="s">
+      <c r="U678" s="6" t="s">
         <v>1186</v>
       </c>
-      <c r="V678" s="1" t="s">
+      <c r="V678" s="6" t="s">
         <v>1187</v>
       </c>
       <c r="W678" s="1" t="s">
@@ -58675,10 +58682,10 @@
       <c r="T679" s="1" t="s">
         <v>672</v>
       </c>
-      <c r="U679" s="1" t="s">
+      <c r="U679" s="6" t="s">
         <v>1190</v>
       </c>
-      <c r="V679" s="1" t="s">
+      <c r="V679" s="6" t="s">
         <v>1191</v>
       </c>
       <c r="W679" s="1" t="s">
@@ -58752,10 +58759,10 @@
       <c r="T680" s="1" t="s">
         <v>1193</v>
       </c>
-      <c r="U680" s="1" t="s">
+      <c r="U680" s="6" t="s">
         <v>1194</v>
       </c>
-      <c r="V680" s="1" t="s">
+      <c r="V680" s="6" t="s">
         <v>1195</v>
       </c>
       <c r="W680" s="1" t="s">
@@ -58829,10 +58836,10 @@
       <c r="T681" s="1" t="s">
         <v>1198</v>
       </c>
-      <c r="U681" s="1" t="s">
+      <c r="U681" s="6" t="s">
         <v>1199</v>
       </c>
-      <c r="V681" s="1" t="s">
+      <c r="V681" s="6" t="s">
         <v>1200</v>
       </c>
       <c r="W681" s="1" t="s">
@@ -58906,10 +58913,10 @@
       <c r="T682" s="1" t="s">
         <v>862</v>
       </c>
-      <c r="U682" s="1" t="s">
+      <c r="U682" s="6" t="s">
         <v>1202</v>
       </c>
-      <c r="V682" s="1" t="s">
+      <c r="V682" s="6" t="s">
         <v>1203</v>
       </c>
       <c r="W682" s="1" t="s">
@@ -58983,10 +58990,10 @@
       <c r="T683" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="U683" s="1" t="s">
+      <c r="U683" s="6" t="s">
         <v>1206</v>
       </c>
-      <c r="V683" s="1" t="s">
+      <c r="V683" s="6" t="s">
         <v>1207</v>
       </c>
       <c r="W683" s="1" t="s">
@@ -59060,10 +59067,10 @@
       <c r="T684" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="U684" s="1" t="s">
+      <c r="U684" s="6" t="s">
         <v>1210</v>
       </c>
-      <c r="V684" s="1" t="s">
+      <c r="V684" s="6" t="s">
         <v>1211</v>
       </c>
       <c r="W684" s="1" t="s">
@@ -59137,10 +59144,10 @@
       <c r="T685" s="1" t="s">
         <v>1214</v>
       </c>
-      <c r="U685" s="1" t="s">
+      <c r="U685" s="6" t="s">
         <v>1215</v>
       </c>
-      <c r="V685" s="1" t="s">
+      <c r="V685" s="6" t="s">
         <v>1216</v>
       </c>
       <c r="W685" s="1" t="s">
@@ -59291,10 +59298,10 @@
       <c r="T687" s="1" t="s">
         <v>1222</v>
       </c>
-      <c r="U687" s="1" t="s">
+      <c r="U687" s="6" t="s">
         <v>1223</v>
       </c>
-      <c r="V687" s="1" t="s">
+      <c r="V687" s="6" t="s">
         <v>1224</v>
       </c>
       <c r="W687" s="1" t="s">
@@ -59445,10 +59452,10 @@
       <c r="T689" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="U689" s="1" t="s">
+      <c r="U689" s="6" t="s">
         <v>1228</v>
       </c>
-      <c r="V689" s="1" t="s">
+      <c r="V689" s="6" t="s">
         <v>1229</v>
       </c>
       <c r="W689" s="1" t="s">
@@ -59522,10 +59529,10 @@
       <c r="T690" s="1" t="s">
         <v>1232</v>
       </c>
-      <c r="U690" s="1" t="s">
+      <c r="U690" s="6" t="s">
         <v>1233</v>
       </c>
-      <c r="V690" s="1" t="s">
+      <c r="V690" s="6" t="s">
         <v>1234</v>
       </c>
       <c r="W690" s="1" t="s">

</xml_diff>